<commit_message>
feat: Enhance BOQ import functionality and update tests
- Added a new route for reviewing BOQ imports.
- Updated the dashboard test to reflect changes in expense titles.
- Modified BOQ completion tests to include new header structure in the imported Excel files.
- Adjusted BOQ import tests to accommodate changes in the workbook structure and validation.
- Improved handling of daywork and percentage adjustments in the BOQ import process.
- Ensured that the import process rejects non-standard BOQ templates.
</commit_message>
<xml_diff>
--- a/resources/templates/boq-import-template.xlsx
+++ b/resources/templates/boq-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ" sheetId="1" r:id="Rc58c798e45754a18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rf264779f937443cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ" sheetId="1" r:id="Rbf2eea13e78e4b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R906b319d9fa74941"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1349,7 +1349,7 @@
         <x:v>Enter items</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
-        <x:v>Fill in the BOQ sheet from row 2. Copy the final row down if you need more than 100 items.</x:v>
+        <x:v>Fill in the BOQ sheet from row 2. Copy the final formatted row down when you need more items.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -1357,7 +1357,7 @@
         <x:v>Reference</x:v>
       </x:c>
       <x:c r="B3" s="13" t="str">
-        <x:v>Keep item references as text, including references such as 12.02(a).</x:v>
+        <x:v>Keep item references as text, including values such as 12.02(a).</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -1365,7 +1365,7 @@
         <x:v>Unit and quantity</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>Use your system unit codes, such as M3, M2 or M. Confirm the unit in the import preview.</x:v>
+        <x:v>Enter the unit and quantity for each item. Use the system unit code where possible. The preview flags units that need attention; no unit conversion is applied.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -1381,7 +1381,7 @@
         <x:v>Amount</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>Quantity multiplied by client rate. Blank rates leave the amount blank. Save in Excel before uploading.</x:v>
+        <x:v>The template calculates quantity multiplied by client rate. Blank rates leave the amount blank. Save in Excel before uploading.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -1389,15 +1389,15 @@
         <x:v>Bills and sections</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>Duplicate the BOQ sheet for another bill. Set bill, section and element for each sheet during import.</x:v>
+        <x:v>Use one BOQ sheet. Add headings such as BILL NO. 1, GROUND FLOOR, ELEMENT NO. 1, or SECTION 8100 in the Description column, leaving Unit and Quantity blank. Items below the heading are grouped under it.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="13" t="str">
-        <x:v>Allowances</x:v>
+        <x:v>Allowances and dayworks</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>Use LS or PS for allowances, normally quantity 1. Confirm the item type and unit in preview.</x:v>
+        <x:v>Use LS or PS for lump sums or provisional sums. Put DAYWORKS on its own heading row to mark following items as dayworks. Complete daywork usage details in the preview.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -1405,7 +1405,7 @@
         <x:v>Upload</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>Select your BOQ sheets and leave Guide unchecked. Start at row 2 and end at the last item.</x:v>
+        <x:v>Keep the sheet named BOQ and keep the six columns in the same order. The optional Guide sheet may remain. Do not add other sheets or change the column headings.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -1413,7 +1413,7 @@
         <x:v>Review</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>Exclude summary totals, VAT, contingency percentages and dayworks. Review the preview, save a draft, then approve it.</x:v>
+        <x:v>Check the item preview, resolve flagged units and daywork details, then save a draft. The approved BOQ changes only after the draft is approved.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>